<commit_message>
Ajout dashboard Ligue 1 et graphiques interactifs
</commit_message>
<xml_diff>
--- a/outputs/dashboard_ligue1.xlsx
+++ b/outputs/dashboard_ligue1.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Data" sheetId="2" state="hidden" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,14 +28,47 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="20"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00666666"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF3F8"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -46,20 +80,42 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -134,6 +190,559 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Points par équipe</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!B45</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$46:$A$63</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$B$46:$B$63</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Points par équipe</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Équipes</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Buts marqués par équipe</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!C45</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$46:$A$63</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$C$46:$C$63</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Buts marqués par équipe</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Équipes</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Clean sheets par équipe</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!D45</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$46:$A$63</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$D$46:$D$63</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Clean sheets par équipe</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Équipes</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>xG par équipe</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!E45</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$46:$A$63</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$E$46:$E$63</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>xG par équipe</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Équipes</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4680000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4680000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4680000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="4680000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -425,161 +1034,964 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE19"/>
+  <dimension ref="A1:L63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Dashboard Ligue 1 - Analyse des facteurs de performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Filtre interactif par catégorie d'équipe : Toutes, Top 5, Milieu ou Bas de tableau</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Catégorie sélectionnée</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Toutes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Meilleure équipe</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Meilleure attaque</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Meilleure défense</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Meilleur buteur</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6">
+        <f>IFERROR(INDEX($A$46:$A$63,MATCH(MAX($B$46:$B$63),$B$46:$B$63,0)),"-")</f>
+        <v/>
+      </c>
+      <c r="D7" s="6">
+        <f>IFERROR(INDEX($A$46:$A$63,MATCH(MAX($C$46:$C$63),$C$46:$C$63,0)),"-")</f>
+        <v/>
+      </c>
+      <c r="G7" s="6">
+        <f>IFERROR(INDEX($A$46:$A$63,MATCH(MIN($F$46:$F$63),$F$46:$F$63,0)),"-")</f>
+        <v/>
+      </c>
+      <c r="J7" s="6">
+        <f>IFERROR(INDEX($G$46:$G$63,MATCH(MAX($H$46:$H$63),$H$46:$H$63,0)),"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Equipe</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Points</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Buts marques</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Clean sheets</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>xG</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>Buts encaisses</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Meilleur buteur</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
+        <is>
+          <t>Buts meilleur buteur</t>
+        </is>
+      </c>
+      <c r="J45">
+        <f>IF($B$4="Toutes",COUNTA(Data!$A$2:$A$19),COUNTIF(Data!$AE$2:$AE$19,$B$4))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <v/>
+      </c>
+      <c r="B46">
+        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <v/>
+      </c>
+      <c r="C46">
+        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <v/>
+      </c>
+      <c r="D46">
+        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <v/>
+      </c>
+      <c r="E46">
+        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <v/>
+      </c>
+      <c r="F46">
+        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <v/>
+      </c>
+      <c r="G46">
+        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <v/>
+      </c>
+      <c r="H46">
+        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <v/>
+      </c>
+      <c r="B47">
+        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <v/>
+      </c>
+      <c r="C47">
+        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <v/>
+      </c>
+      <c r="D47">
+        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <v/>
+      </c>
+      <c r="E47">
+        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <v/>
+      </c>
+      <c r="F47">
+        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <v/>
+      </c>
+      <c r="G47">
+        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <v/>
+      </c>
+      <c r="H47">
+        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <v/>
+      </c>
+      <c r="B48">
+        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <v/>
+      </c>
+      <c r="C48">
+        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <v/>
+      </c>
+      <c r="D48">
+        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <v/>
+      </c>
+      <c r="E48">
+        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <v/>
+      </c>
+      <c r="F48">
+        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <v/>
+      </c>
+      <c r="G48">
+        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <v/>
+      </c>
+      <c r="H48">
+        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <v/>
+      </c>
+      <c r="B49">
+        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <v/>
+      </c>
+      <c r="C49">
+        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <v/>
+      </c>
+      <c r="D49">
+        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <v/>
+      </c>
+      <c r="E49">
+        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <v/>
+      </c>
+      <c r="F49">
+        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <v/>
+      </c>
+      <c r="G49">
+        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <v/>
+      </c>
+      <c r="H49">
+        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <v/>
+      </c>
+      <c r="B50">
+        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <v/>
+      </c>
+      <c r="C50">
+        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <v/>
+      </c>
+      <c r="D50">
+        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <v/>
+      </c>
+      <c r="E50">
+        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <v/>
+      </c>
+      <c r="F50">
+        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <v/>
+      </c>
+      <c r="G50">
+        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <v/>
+      </c>
+      <c r="H50">
+        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <v/>
+      </c>
+      <c r="B51">
+        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <v/>
+      </c>
+      <c r="C51">
+        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <v/>
+      </c>
+      <c r="D51">
+        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <v/>
+      </c>
+      <c r="E51">
+        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <v/>
+      </c>
+      <c r="F51">
+        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <v/>
+      </c>
+      <c r="G51">
+        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <v/>
+      </c>
+      <c r="H51">
+        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <v/>
+      </c>
+      <c r="B52">
+        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <v/>
+      </c>
+      <c r="C52">
+        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <v/>
+      </c>
+      <c r="D52">
+        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <v/>
+      </c>
+      <c r="E52">
+        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <v/>
+      </c>
+      <c r="F52">
+        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <v/>
+      </c>
+      <c r="G52">
+        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <v/>
+      </c>
+      <c r="H52">
+        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <v/>
+      </c>
+      <c r="B53">
+        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <v/>
+      </c>
+      <c r="C53">
+        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <v/>
+      </c>
+      <c r="D53">
+        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <v/>
+      </c>
+      <c r="E53">
+        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <v/>
+      </c>
+      <c r="F53">
+        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <v/>
+      </c>
+      <c r="G53">
+        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <v/>
+      </c>
+      <c r="H53">
+        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <v/>
+      </c>
+      <c r="B54">
+        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <v/>
+      </c>
+      <c r="C54">
+        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <v/>
+      </c>
+      <c r="D54">
+        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <v/>
+      </c>
+      <c r="E54">
+        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <v/>
+      </c>
+      <c r="F54">
+        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <v/>
+      </c>
+      <c r="G54">
+        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <v/>
+      </c>
+      <c r="H54">
+        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <v/>
+      </c>
+      <c r="B55">
+        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <v/>
+      </c>
+      <c r="C55">
+        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <v/>
+      </c>
+      <c r="D55">
+        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <v/>
+      </c>
+      <c r="E55">
+        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <v/>
+      </c>
+      <c r="F55">
+        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <v/>
+      </c>
+      <c r="G55">
+        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <v/>
+      </c>
+      <c r="H55">
+        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <v/>
+      </c>
+      <c r="B56">
+        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <v/>
+      </c>
+      <c r="C56">
+        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <v/>
+      </c>
+      <c r="D56">
+        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <v/>
+      </c>
+      <c r="E56">
+        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <v/>
+      </c>
+      <c r="F56">
+        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <v/>
+      </c>
+      <c r="G56">
+        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <v/>
+      </c>
+      <c r="H56">
+        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <v/>
+      </c>
+      <c r="B57">
+        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <v/>
+      </c>
+      <c r="C57">
+        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <v/>
+      </c>
+      <c r="D57">
+        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <v/>
+      </c>
+      <c r="E57">
+        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <v/>
+      </c>
+      <c r="F57">
+        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <v/>
+      </c>
+      <c r="G57">
+        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <v/>
+      </c>
+      <c r="H57">
+        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <v/>
+      </c>
+      <c r="B58">
+        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <v/>
+      </c>
+      <c r="C58">
+        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <v/>
+      </c>
+      <c r="D58">
+        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <v/>
+      </c>
+      <c r="E58">
+        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <v/>
+      </c>
+      <c r="F58">
+        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <v/>
+      </c>
+      <c r="G58">
+        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <v/>
+      </c>
+      <c r="H58">
+        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <v/>
+      </c>
+      <c r="B59">
+        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <v/>
+      </c>
+      <c r="C59">
+        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <v/>
+      </c>
+      <c r="D59">
+        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <v/>
+      </c>
+      <c r="E59">
+        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <v/>
+      </c>
+      <c r="F59">
+        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <v/>
+      </c>
+      <c r="G59">
+        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <v/>
+      </c>
+      <c r="H59">
+        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <v/>
+      </c>
+      <c r="B60">
+        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <v/>
+      </c>
+      <c r="C60">
+        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <v/>
+      </c>
+      <c r="D60">
+        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <v/>
+      </c>
+      <c r="E60">
+        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <v/>
+      </c>
+      <c r="F60">
+        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <v/>
+      </c>
+      <c r="G60">
+        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <v/>
+      </c>
+      <c r="H60">
+        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <v/>
+      </c>
+      <c r="B61">
+        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <v/>
+      </c>
+      <c r="C61">
+        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <v/>
+      </c>
+      <c r="D61">
+        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <v/>
+      </c>
+      <c r="E61">
+        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <v/>
+      </c>
+      <c r="F61">
+        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <v/>
+      </c>
+      <c r="G61">
+        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <v/>
+      </c>
+      <c r="H61">
+        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <v/>
+      </c>
+      <c r="B62">
+        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <v/>
+      </c>
+      <c r="C62">
+        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <v/>
+      </c>
+      <c r="D62">
+        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <v/>
+      </c>
+      <c r="E62">
+        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <v/>
+      </c>
+      <c r="F62">
+        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <v/>
+      </c>
+      <c r="G62">
+        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <v/>
+      </c>
+      <c r="H62">
+        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <v/>
+      </c>
+      <c r="B63">
+        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <v/>
+      </c>
+      <c r="C63">
+        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <v/>
+      </c>
+      <c r="D63">
+        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <v/>
+      </c>
+      <c r="E63">
+        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <v/>
+      </c>
+      <c r="F63">
+        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <v/>
+      </c>
+      <c r="G63">
+        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <v/>
+      </c>
+      <c r="H63">
+        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="A6:B6"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Toutes,Top 5,Milieu,Bas de tableau"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AE19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
+    <col width="18" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="18" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="18" customWidth="1" min="25" max="25"/>
+    <col width="18" customWidth="1" min="26" max="26"/>
+    <col width="18" customWidth="1" min="27" max="27"/>
+    <col width="18" customWidth="1" min="28" max="28"/>
+    <col width="18" customWidth="1" min="29" max="29"/>
+    <col width="18" customWidth="1" min="30" max="30"/>
+    <col width="18" customWidth="1" min="31" max="31"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
           <t>equipe</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>rang</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>journees</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>points</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>victoires</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>nuls</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>defaites</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>buts_marques</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>buts_encaisses</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>difference_buts</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>points_domicile</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>points_exterieur</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>victoires_domicile</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>victoires_exterieur</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>buts_domicile</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>buts_exterieur</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>clean_sheets</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>possession_moyenne</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>tirs_par_match</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>xG</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>xGA</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>cartons_jaunes</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>cartons_rouges</t>
         </is>
       </c>
-      <c r="X1" s="1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>meilleur_buteur</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>buts_meilleur_buteur</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>meilleur_passeur</t>
         </is>
       </c>
-      <c r="AA1" s="1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>passes_decisives</t>
         </is>
       </c>
-      <c r="AB1" s="1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>efficacite_offensive</t>
         </is>
       </c>
-      <c r="AC1" s="1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>solidite_defensive</t>
         </is>
       </c>
-      <c r="AD1" s="1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>indice_discipline</t>
         </is>
       </c>
-      <c r="AE1" s="1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>categorie_equipe</t>
         </is>

</xml_diff>

<commit_message>
Ajout page analyse avancee et amelioration dashboard
</commit_message>
<xml_diff>
--- a/outputs/dashboard_ligue1.xlsx
+++ b/outputs/dashboard_ligue1.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Data" sheetId="2" state="hidden" r:id="rId2"/>
+    <sheet name="Analyse_avancee" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -652,6 +653,488 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Efficacité offensive</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Analyse_avancee'!B5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Analyse_avancee'!$A$6:$A$23</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Analyse_avancee'!$B$6:$B$23</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Efficacité offensive</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Équipes</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Buts encaissés</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Analyse_avancee'!F5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Analyse_avancee'!$E$6:$E$23</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Analyse_avancee'!$F$6:$F$23</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Buts encaissés</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Équipes</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Indice discipline</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Analyse_avancee'!B25</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Analyse_avancee'!$A$26:$A$43</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Analyse_avancee'!$B$26:$B$43</f>
+            </numRef>
+          </val>
+        </ser>
+        <dLbls>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Indice discipline</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Équipes</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart8.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Points domicile vs extérieur</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Analyse_avancee'!F25</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Analyse_avancee'!$E$26:$E$43</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Analyse_avancee'!$F$26:$F$43</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Analyse_avancee'!G25</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Analyse_avancee'!$E$26:$E$43</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Analyse_avancee'!$G$26:$G$43</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Points</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Équipes</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -659,6 +1142,99 @@
       <col>0</col>
       <colOff>0</colOff>
       <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>9</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>7</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4680000" cy="2880000"/>
@@ -680,7 +1256,7 @@
     <from>
       <col>6</col>
       <colOff>0</colOff>
-      <row>9</row>
+      <row>7</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4680000" cy="2880000"/>
@@ -1158,620 +1734,616 @@
           <t>Buts meilleur buteur</t>
         </is>
       </c>
-      <c r="J45">
-        <f>IF($B$4="Toutes",COUNTA(Data!$A$2:$A$19),COUNTIF(Data!$AE$2:$AE$19,$B$4))</f>
-        <v/>
-      </c>
     </row>
     <row r="46">
       <c r="A46">
-        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!A2,"")</f>
         <v/>
       </c>
       <c r="B46">
-        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!D2,"")</f>
         <v/>
       </c>
       <c r="C46">
-        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!H2,"")</f>
         <v/>
       </c>
       <c r="D46">
-        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!Q2,"")</f>
         <v/>
       </c>
       <c r="E46">
-        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!T2,NA())</f>
         <v/>
       </c>
       <c r="F46">
-        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!I2,999)</f>
         <v/>
       </c>
       <c r="G46">
-        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!X2,"")</f>
         <v/>
       </c>
       <c r="H46">
-        <f>IF(ROWS($A$46:A46)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),1)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!Y2,0)</f>
         <v/>
       </c>
     </row>
     <row r="47">
       <c r="A47">
-        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!A3,"")</f>
         <v/>
       </c>
       <c r="B47">
-        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!D3,"")</f>
         <v/>
       </c>
       <c r="C47">
-        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!H3,"")</f>
         <v/>
       </c>
       <c r="D47">
-        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!Q3,"")</f>
         <v/>
       </c>
       <c r="E47">
-        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!T3,NA())</f>
         <v/>
       </c>
       <c r="F47">
-        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!I3,999)</f>
         <v/>
       </c>
       <c r="G47">
-        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!X3,"")</f>
         <v/>
       </c>
       <c r="H47">
-        <f>IF(ROWS($A$46:A47)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),2)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!Y3,0)</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48">
-        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!A4,"")</f>
         <v/>
       </c>
       <c r="B48">
-        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!D4,"")</f>
         <v/>
       </c>
       <c r="C48">
-        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!H4,"")</f>
         <v/>
       </c>
       <c r="D48">
-        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!Q4,"")</f>
         <v/>
       </c>
       <c r="E48">
-        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!T4,NA())</f>
         <v/>
       </c>
       <c r="F48">
-        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!I4,999)</f>
         <v/>
       </c>
       <c r="G48">
-        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!X4,"")</f>
         <v/>
       </c>
       <c r="H48">
-        <f>IF(ROWS($A$46:A48)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),3)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!Y4,0)</f>
         <v/>
       </c>
     </row>
     <row r="49">
       <c r="A49">
-        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!A5,"")</f>
         <v/>
       </c>
       <c r="B49">
-        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!D5,"")</f>
         <v/>
       </c>
       <c r="C49">
-        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!H5,"")</f>
         <v/>
       </c>
       <c r="D49">
-        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!Q5,"")</f>
         <v/>
       </c>
       <c r="E49">
-        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!T5,NA())</f>
         <v/>
       </c>
       <c r="F49">
-        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!I5,999)</f>
         <v/>
       </c>
       <c r="G49">
-        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!X5,"")</f>
         <v/>
       </c>
       <c r="H49">
-        <f>IF(ROWS($A$46:A49)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),4)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!Y5,0)</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50">
-        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!A6,"")</f>
         <v/>
       </c>
       <c r="B50">
-        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!D6,"")</f>
         <v/>
       </c>
       <c r="C50">
-        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!H6,"")</f>
         <v/>
       </c>
       <c r="D50">
-        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!Q6,"")</f>
         <v/>
       </c>
       <c r="E50">
-        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!T6,NA())</f>
         <v/>
       </c>
       <c r="F50">
-        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!I6,999)</f>
         <v/>
       </c>
       <c r="G50">
-        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!X6,"")</f>
         <v/>
       </c>
       <c r="H50">
-        <f>IF(ROWS($A$46:A50)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),5)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!Y6,0)</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51">
-        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!A7,"")</f>
         <v/>
       </c>
       <c r="B51">
-        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!D7,"")</f>
         <v/>
       </c>
       <c r="C51">
-        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!H7,"")</f>
         <v/>
       </c>
       <c r="D51">
-        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!Q7,"")</f>
         <v/>
       </c>
       <c r="E51">
-        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!T7,NA())</f>
         <v/>
       </c>
       <c r="F51">
-        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!I7,999)</f>
         <v/>
       </c>
       <c r="G51">
-        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!X7,"")</f>
         <v/>
       </c>
       <c r="H51">
-        <f>IF(ROWS($A$46:A51)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),6)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!Y7,0)</f>
         <v/>
       </c>
     </row>
     <row r="52">
       <c r="A52">
-        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!A8,"")</f>
         <v/>
       </c>
       <c r="B52">
-        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!D8,"")</f>
         <v/>
       </c>
       <c r="C52">
-        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!H8,"")</f>
         <v/>
       </c>
       <c r="D52">
-        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!Q8,"")</f>
         <v/>
       </c>
       <c r="E52">
-        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!T8,NA())</f>
         <v/>
       </c>
       <c r="F52">
-        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!I8,999)</f>
         <v/>
       </c>
       <c r="G52">
-        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!X8,"")</f>
         <v/>
       </c>
       <c r="H52">
-        <f>IF(ROWS($A$46:A52)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),7)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!Y8,0)</f>
         <v/>
       </c>
     </row>
     <row r="53">
       <c r="A53">
-        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!A9,"")</f>
         <v/>
       </c>
       <c r="B53">
-        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!D9,"")</f>
         <v/>
       </c>
       <c r="C53">
-        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!H9,"")</f>
         <v/>
       </c>
       <c r="D53">
-        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!Q9,"")</f>
         <v/>
       </c>
       <c r="E53">
-        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!T9,NA())</f>
         <v/>
       </c>
       <c r="F53">
-        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!I9,999)</f>
         <v/>
       </c>
       <c r="G53">
-        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!X9,"")</f>
         <v/>
       </c>
       <c r="H53">
-        <f>IF(ROWS($A$46:A53)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),8)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!Y9,0)</f>
         <v/>
       </c>
     </row>
     <row r="54">
       <c r="A54">
-        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!A10,"")</f>
         <v/>
       </c>
       <c r="B54">
-        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!D10,"")</f>
         <v/>
       </c>
       <c r="C54">
-        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!H10,"")</f>
         <v/>
       </c>
       <c r="D54">
-        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!Q10,"")</f>
         <v/>
       </c>
       <c r="E54">
-        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!T10,NA())</f>
         <v/>
       </c>
       <c r="F54">
-        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!I10,999)</f>
         <v/>
       </c>
       <c r="G54">
-        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!X10,"")</f>
         <v/>
       </c>
       <c r="H54">
-        <f>IF(ROWS($A$46:A54)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),9)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!Y10,0)</f>
         <v/>
       </c>
     </row>
     <row r="55">
       <c r="A55">
-        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!A11,"")</f>
         <v/>
       </c>
       <c r="B55">
-        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!D11,"")</f>
         <v/>
       </c>
       <c r="C55">
-        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!H11,"")</f>
         <v/>
       </c>
       <c r="D55">
-        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!Q11,"")</f>
         <v/>
       </c>
       <c r="E55">
-        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!T11,NA())</f>
         <v/>
       </c>
       <c r="F55">
-        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!I11,999)</f>
         <v/>
       </c>
       <c r="G55">
-        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!X11,"")</f>
         <v/>
       </c>
       <c r="H55">
-        <f>IF(ROWS($A$46:A55)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),10)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!Y11,0)</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56">
-        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!A12,"")</f>
         <v/>
       </c>
       <c r="B56">
-        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!D12,"")</f>
         <v/>
       </c>
       <c r="C56">
-        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!H12,"")</f>
         <v/>
       </c>
       <c r="D56">
-        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!Q12,"")</f>
         <v/>
       </c>
       <c r="E56">
-        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!T12,NA())</f>
         <v/>
       </c>
       <c r="F56">
-        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!I12,999)</f>
         <v/>
       </c>
       <c r="G56">
-        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!X12,"")</f>
         <v/>
       </c>
       <c r="H56">
-        <f>IF(ROWS($A$46:A56)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),11)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!Y12,0)</f>
         <v/>
       </c>
     </row>
     <row r="57">
       <c r="A57">
-        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!A13,"")</f>
         <v/>
       </c>
       <c r="B57">
-        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!D13,"")</f>
         <v/>
       </c>
       <c r="C57">
-        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!H13,"")</f>
         <v/>
       </c>
       <c r="D57">
-        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!Q13,"")</f>
         <v/>
       </c>
       <c r="E57">
-        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!T13,NA())</f>
         <v/>
       </c>
       <c r="F57">
-        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!I13,999)</f>
         <v/>
       </c>
       <c r="G57">
-        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!X13,"")</f>
         <v/>
       </c>
       <c r="H57">
-        <f>IF(ROWS($A$46:A57)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),12)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!Y13,0)</f>
         <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58">
-        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!A14,"")</f>
         <v/>
       </c>
       <c r="B58">
-        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!D14,"")</f>
         <v/>
       </c>
       <c r="C58">
-        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!H14,"")</f>
         <v/>
       </c>
       <c r="D58">
-        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!Q14,"")</f>
         <v/>
       </c>
       <c r="E58">
-        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!T14,NA())</f>
         <v/>
       </c>
       <c r="F58">
-        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!I14,999)</f>
         <v/>
       </c>
       <c r="G58">
-        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!X14,"")</f>
         <v/>
       </c>
       <c r="H58">
-        <f>IF(ROWS($A$46:A58)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),13)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!Y14,0)</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59">
-        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!A15,"")</f>
         <v/>
       </c>
       <c r="B59">
-        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!D15,"")</f>
         <v/>
       </c>
       <c r="C59">
-        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!H15,"")</f>
         <v/>
       </c>
       <c r="D59">
-        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!Q15,"")</f>
         <v/>
       </c>
       <c r="E59">
-        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!T15,NA())</f>
         <v/>
       </c>
       <c r="F59">
-        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!I15,999)</f>
         <v/>
       </c>
       <c r="G59">
-        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!X15,"")</f>
         <v/>
       </c>
       <c r="H59">
-        <f>IF(ROWS($A$46:A59)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),14)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!Y15,0)</f>
         <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60">
-        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!A16,"")</f>
         <v/>
       </c>
       <c r="B60">
-        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!D16,"")</f>
         <v/>
       </c>
       <c r="C60">
-        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!H16,"")</f>
         <v/>
       </c>
       <c r="D60">
-        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!Q16,"")</f>
         <v/>
       </c>
       <c r="E60">
-        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!T16,NA())</f>
         <v/>
       </c>
       <c r="F60">
-        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!I16,999)</f>
         <v/>
       </c>
       <c r="G60">
-        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!X16,"")</f>
         <v/>
       </c>
       <c r="H60">
-        <f>IF(ROWS($A$46:A60)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),15)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!Y16,0)</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61">
-        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!A17,"")</f>
         <v/>
       </c>
       <c r="B61">
-        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!D17,"")</f>
         <v/>
       </c>
       <c r="C61">
-        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!H17,"")</f>
         <v/>
       </c>
       <c r="D61">
-        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!Q17,"")</f>
         <v/>
       </c>
       <c r="E61">
-        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!T17,NA())</f>
         <v/>
       </c>
       <c r="F61">
-        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!I17,999)</f>
         <v/>
       </c>
       <c r="G61">
-        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!X17,"")</f>
         <v/>
       </c>
       <c r="H61">
-        <f>IF(ROWS($A$46:A61)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),16)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!Y17,0)</f>
         <v/>
       </c>
     </row>
     <row r="62">
       <c r="A62">
-        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!A18,"")</f>
         <v/>
       </c>
       <c r="B62">
-        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!D18,"")</f>
         <v/>
       </c>
       <c r="C62">
-        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!H18,"")</f>
         <v/>
       </c>
       <c r="D62">
-        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!Q18,"")</f>
         <v/>
       </c>
       <c r="E62">
-        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!T18,NA())</f>
         <v/>
       </c>
       <c r="F62">
-        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!I18,999)</f>
         <v/>
       </c>
       <c r="G62">
-        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!X18,"")</f>
         <v/>
       </c>
       <c r="H62">
-        <f>IF(ROWS($A$46:A62)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),17)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!Y18,0)</f>
         <v/>
       </c>
     </row>
     <row r="63">
       <c r="A63">
-        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$A$2:$A$19,AGGREGATE(15,6,(ROW(Data!$A$2:$A$19)-ROW(Data!$A$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!A19,"")</f>
         <v/>
       </c>
       <c r="B63">
-        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$D$2:$D$19,AGGREGATE(15,6,(ROW(Data!$D$2:$D$19)-ROW(Data!$D$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!D19,"")</f>
         <v/>
       </c>
       <c r="C63">
-        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$H$2:$H$19,AGGREGATE(15,6,(ROW(Data!$H$2:$H$19)-ROW(Data!$H$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!H19,"")</f>
         <v/>
       </c>
       <c r="D63">
-        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$Q$2:$Q$19,AGGREGATE(15,6,(ROW(Data!$Q$2:$Q$19)-ROW(Data!$Q$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!Q19,"")</f>
         <v/>
       </c>
       <c r="E63">
-        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$T$2:$T$19,AGGREGATE(15,6,(ROW(Data!$T$2:$T$19)-ROW(Data!$T$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!T19,NA())</f>
         <v/>
       </c>
       <c r="F63">
-        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$I$2:$I$19,AGGREGATE(15,6,(ROW(Data!$I$2:$I$19)-ROW(Data!$I$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!I19,999)</f>
         <v/>
       </c>
       <c r="G63">
-        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$X$2:$X$19,AGGREGATE(15,6,(ROW(Data!$X$2:$X$19)-ROW(Data!$X$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!X19,"")</f>
         <v/>
       </c>
       <c r="H63">
-        <f>IF(ROWS($A$46:A63)&gt;$J$45,"",INDEX(Data!$Y$2:$Y$19,AGGREGATE(15,6,(ROW(Data!$Y$2:$Y$19)-ROW(Data!$Y$2)+1)/IF($B$4="Toutes",1,(Data!$AE$2:$AE$19=$B$4)),18)))</f>
+        <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!Y19,0)</f>
         <v/>
       </c>
     </row>
@@ -3854,4 +4426,802 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Analyse avancée - Ligue 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Analyse complémentaire : efficacité offensive, défense, discipline et domicile/extérieur</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>equipe</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>efficacite_offensive</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>equipe</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>buts_encaisses</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>PSG</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>PSG</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Lille</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Marseille</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Nice</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Marseille</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Lorient</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Lille</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Strasbourg</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Nice</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Brest</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Toulouse</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Brest</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Auxerre</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Auxerre</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Toulouse</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Strasbourg</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Angers</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Metz</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Le Havre</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Angers</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Lorient</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Le Havre</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Metz</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Paris FC</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Paris FC</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="7" t="inlineStr">
+        <is>
+          <t>equipe</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>indice_discipline</t>
+        </is>
+      </c>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>equipe</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr">
+        <is>
+          <t>points_domicile</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>points_exterieur</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Paris FC</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>100</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>PSG</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>43</v>
+      </c>
+      <c r="G26" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Metz</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>95</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Lille</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>35</v>
+      </c>
+      <c r="G27" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Lorient</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>94</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Nice</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>34</v>
+      </c>
+      <c r="G28" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Le Havre</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>91</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Marseille</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>32</v>
+      </c>
+      <c r="G29" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Auxerre</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>85</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>31</v>
+      </c>
+      <c r="G30" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>85</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>31</v>
+      </c>
+      <c r="G31" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Angers</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>84</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Strasbourg</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>30</v>
+      </c>
+      <c r="G32" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>82</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>28</v>
+      </c>
+      <c r="G33" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Rennes</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>80</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Lyon</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>26</v>
+      </c>
+      <c r="G34" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Strasbourg</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>78</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Toulouse</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>26</v>
+      </c>
+      <c r="G35" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Lens</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>77</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Auxerre</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>25</v>
+      </c>
+      <c r="G36" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Marseille</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>73</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Brest</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>22</v>
+      </c>
+      <c r="G37" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Toulouse</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>73</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Angers</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>22</v>
+      </c>
+      <c r="G38" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Nice</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>72</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Le Havre</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>21</v>
+      </c>
+      <c r="G39" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Brest</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>71</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Lorient</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>20</v>
+      </c>
+      <c r="G40" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Monaco</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>67</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Nantes</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>18</v>
+      </c>
+      <c r="G41" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>PSG</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>64</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Metz</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>18</v>
+      </c>
+      <c r="G42" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Lille</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>60</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Paris FC</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>16</v>
+      </c>
+      <c r="G43" t="n">
+        <v>12</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Sauvegarde avant restructuration uv
</commit_message>
<xml_diff>
--- a/outputs/dashboard_ligue1.xlsx
+++ b/outputs/dashboard_ligue1.xlsx
@@ -221,7 +221,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!B45</f>
+              <f>'Dashboard'!B90</f>
             </strRef>
           </tx>
           <spPr>
@@ -231,12 +231,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$46:$A$63</f>
+              <f>'Dashboard'!$A$91:$A$108</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$B$46:$B$63</f>
+              <f>'Dashboard'!$B$91:$B$108</f>
             </numRef>
           </val>
         </ser>
@@ -336,7 +336,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!C45</f>
+              <f>'Dashboard'!C90</f>
             </strRef>
           </tx>
           <spPr>
@@ -346,12 +346,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$46:$A$63</f>
+              <f>'Dashboard'!$A$91:$A$108</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$C$46:$C$63</f>
+              <f>'Dashboard'!$C$91:$C$108</f>
             </numRef>
           </val>
         </ser>
@@ -451,7 +451,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!D45</f>
+              <f>'Dashboard'!D90</f>
             </strRef>
           </tx>
           <spPr>
@@ -461,12 +461,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$46:$A$63</f>
+              <f>'Dashboard'!$A$91:$A$108</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$D$46:$D$63</f>
+              <f>'Dashboard'!$D$91:$D$108</f>
             </numRef>
           </val>
         </ser>
@@ -566,7 +566,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Dashboard'!E45</f>
+              <f>'Dashboard'!E90</f>
             </strRef>
           </tx>
           <spPr>
@@ -576,12 +576,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Dashboard'!$A$46:$A$63</f>
+              <f>'Dashboard'!$A$91:$A$108</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Dashboard'!$E$46:$E$63</f>
+              <f>'Dashboard'!$E$91:$E$108</f>
             </numRef>
           </val>
         </ser>
@@ -681,7 +681,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Analyse_avancee'!B5</f>
+              <f>'Analyse_avancee'!B60</f>
             </strRef>
           </tx>
           <spPr>
@@ -691,12 +691,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Analyse_avancee'!$A$6:$A$23</f>
+              <f>'Analyse_avancee'!$A$61:$A$78</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Analyse_avancee'!$B$6:$B$23</f>
+              <f>'Analyse_avancee'!$B$61:$B$78</f>
             </numRef>
           </val>
         </ser>
@@ -796,7 +796,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Analyse_avancee'!F5</f>
+              <f>'Analyse_avancee'!F60</f>
             </strRef>
           </tx>
           <spPr>
@@ -806,12 +806,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Analyse_avancee'!$E$6:$E$23</f>
+              <f>'Analyse_avancee'!$E$61:$E$78</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Analyse_avancee'!$F$6:$F$23</f>
+              <f>'Analyse_avancee'!$F$61:$F$78</f>
             </numRef>
           </val>
         </ser>
@@ -911,7 +911,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Analyse_avancee'!B25</f>
+              <f>'Analyse_avancee'!B85</f>
             </strRef>
           </tx>
           <spPr>
@@ -921,12 +921,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Analyse_avancee'!$A$26:$A$43</f>
+              <f>'Analyse_avancee'!$A$86:$A$103</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Analyse_avancee'!$B$26:$B$43</f>
+              <f>'Analyse_avancee'!$B$86:$B$103</f>
             </numRef>
           </val>
         </ser>
@@ -1026,7 +1026,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Analyse_avancee'!F25</f>
+              <f>'Analyse_avancee'!F85</f>
             </strRef>
           </tx>
           <spPr>
@@ -1036,12 +1036,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Analyse_avancee'!$E$26:$E$43</f>
+              <f>'Analyse_avancee'!$E$86:$E$103</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Analyse_avancee'!$F$26:$F$43</f>
+              <f>'Analyse_avancee'!$F$86:$F$103</f>
             </numRef>
           </val>
         </ser>
@@ -1050,7 +1050,7 @@
           <order val="1"/>
           <tx>
             <strRef>
-              <f>'Analyse_avancee'!G25</f>
+              <f>'Analyse_avancee'!G85</f>
             </strRef>
           </tx>
           <spPr>
@@ -1060,12 +1060,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Analyse_avancee'!$E$26:$E$43</f>
+              <f>'Analyse_avancee'!$E$86:$E$103</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Analyse_avancee'!$G$26:$G$43</f>
+              <f>'Analyse_avancee'!$G$86:$G$103</f>
             </numRef>
           </val>
         </ser>
@@ -1300,7 +1300,7 @@
     <from>
       <col>6</col>
       <colOff>0</colOff>
-      <row>27</row>
+      <row>24</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="4680000" cy="2880000"/>
@@ -1610,7 +1610,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L63"/>
+  <dimension ref="A1:L108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1677,672 +1677,672 @@
     </row>
     <row r="7">
       <c r="A7" s="6">
-        <f>IFERROR(INDEX($A$46:$A$63,MATCH(MAX($B$46:$B$63),$B$46:$B$63,0)),"-")</f>
+        <f>IFERROR(INDEX($A$91:$A$108,MATCH(MAX($B$91:$B$108),$B$91:$B$108,0)),"-")</f>
         <v/>
       </c>
       <c r="D7" s="6">
-        <f>IFERROR(INDEX($A$46:$A$63,MATCH(MAX($C$46:$C$63),$C$46:$C$63,0)),"-")</f>
+        <f>IFERROR(INDEX($A$91:$A$108,MATCH(MAX($C$91:$C$108),$C$91:$C$108,0)),"-")</f>
         <v/>
       </c>
       <c r="G7" s="6">
-        <f>IFERROR(INDEX($A$46:$A$63,MATCH(MIN($F$46:$F$63),$F$46:$F$63,0)),"-")</f>
+        <f>IFERROR(INDEX($A$91:$A$108,MATCH(MIN($F$91:$F$108),$F$91:$F$108,0)),"-")</f>
         <v/>
       </c>
       <c r="J7" s="6">
-        <f>IFERROR(INDEX($G$46:$G$63,MATCH(MAX($H$46:$H$63),$H$46:$H$63,0)),"-")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="7" t="inlineStr">
+        <f>IFERROR(INDEX($G$91:$G$108,MATCH(MAX($H$91:$H$108),$H$91:$H$108,0)),"-")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="7" t="inlineStr">
         <is>
           <t>Equipe</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr">
+      <c r="B90" s="7" t="inlineStr">
         <is>
           <t>Points</t>
         </is>
       </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C90" s="7" t="inlineStr">
         <is>
           <t>Buts marques</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D90" s="7" t="inlineStr">
         <is>
           <t>Clean sheets</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
+      <c r="E90" s="7" t="inlineStr">
         <is>
           <t>xG</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
+      <c r="F90" s="7" t="inlineStr">
         <is>
           <t>Buts encaisses</t>
         </is>
       </c>
-      <c r="G45" s="7" t="inlineStr">
+      <c r="G90" s="7" t="inlineStr">
         <is>
           <t>Meilleur buteur</t>
         </is>
       </c>
-      <c r="H45" s="7" t="inlineStr">
+      <c r="H90" s="7" t="inlineStr">
         <is>
           <t>Buts meilleur buteur</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46">
+    <row r="91">
+      <c r="A91">
         <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!A2,"")</f>
         <v/>
       </c>
-      <c r="B46">
+      <c r="B91">
         <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!D2,"")</f>
         <v/>
       </c>
-      <c r="C46">
+      <c r="C91">
         <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!H2,"")</f>
         <v/>
       </c>
-      <c r="D46">
+      <c r="D91">
         <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!Q2,"")</f>
         <v/>
       </c>
-      <c r="E46">
+      <c r="E91">
         <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!T2,NA())</f>
         <v/>
       </c>
-      <c r="F46">
+      <c r="F91">
         <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!I2,999)</f>
         <v/>
       </c>
-      <c r="G46">
+      <c r="G91">
         <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!X2,"")</f>
         <v/>
       </c>
-      <c r="H46">
+      <c r="H91">
         <f>IF(OR($B$4="Toutes",Data!AE2=$B$4),Data!Y2,0)</f>
         <v/>
       </c>
     </row>
-    <row r="47">
-      <c r="A47">
+    <row r="92">
+      <c r="A92">
         <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!A3,"")</f>
         <v/>
       </c>
-      <c r="B47">
+      <c r="B92">
         <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!D3,"")</f>
         <v/>
       </c>
-      <c r="C47">
+      <c r="C92">
         <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!H3,"")</f>
         <v/>
       </c>
-      <c r="D47">
+      <c r="D92">
         <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!Q3,"")</f>
         <v/>
       </c>
-      <c r="E47">
+      <c r="E92">
         <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!T3,NA())</f>
         <v/>
       </c>
-      <c r="F47">
+      <c r="F92">
         <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!I3,999)</f>
         <v/>
       </c>
-      <c r="G47">
+      <c r="G92">
         <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!X3,"")</f>
         <v/>
       </c>
-      <c r="H47">
+      <c r="H92">
         <f>IF(OR($B$4="Toutes",Data!AE3=$B$4),Data!Y3,0)</f>
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48">
+    <row r="93">
+      <c r="A93">
         <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!A4,"")</f>
         <v/>
       </c>
-      <c r="B48">
+      <c r="B93">
         <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!D4,"")</f>
         <v/>
       </c>
-      <c r="C48">
+      <c r="C93">
         <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!H4,"")</f>
         <v/>
       </c>
-      <c r="D48">
+      <c r="D93">
         <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!Q4,"")</f>
         <v/>
       </c>
-      <c r="E48">
+      <c r="E93">
         <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!T4,NA())</f>
         <v/>
       </c>
-      <c r="F48">
+      <c r="F93">
         <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!I4,999)</f>
         <v/>
       </c>
-      <c r="G48">
+      <c r="G93">
         <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!X4,"")</f>
         <v/>
       </c>
-      <c r="H48">
+      <c r="H93">
         <f>IF(OR($B$4="Toutes",Data!AE4=$B$4),Data!Y4,0)</f>
         <v/>
       </c>
     </row>
-    <row r="49">
-      <c r="A49">
+    <row r="94">
+      <c r="A94">
         <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!A5,"")</f>
         <v/>
       </c>
-      <c r="B49">
+      <c r="B94">
         <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!D5,"")</f>
         <v/>
       </c>
-      <c r="C49">
+      <c r="C94">
         <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!H5,"")</f>
         <v/>
       </c>
-      <c r="D49">
+      <c r="D94">
         <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!Q5,"")</f>
         <v/>
       </c>
-      <c r="E49">
+      <c r="E94">
         <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!T5,NA())</f>
         <v/>
       </c>
-      <c r="F49">
+      <c r="F94">
         <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!I5,999)</f>
         <v/>
       </c>
-      <c r="G49">
+      <c r="G94">
         <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!X5,"")</f>
         <v/>
       </c>
-      <c r="H49">
+      <c r="H94">
         <f>IF(OR($B$4="Toutes",Data!AE5=$B$4),Data!Y5,0)</f>
         <v/>
       </c>
     </row>
-    <row r="50">
-      <c r="A50">
+    <row r="95">
+      <c r="A95">
         <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!A6,"")</f>
         <v/>
       </c>
-      <c r="B50">
+      <c r="B95">
         <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!D6,"")</f>
         <v/>
       </c>
-      <c r="C50">
+      <c r="C95">
         <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!H6,"")</f>
         <v/>
       </c>
-      <c r="D50">
+      <c r="D95">
         <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!Q6,"")</f>
         <v/>
       </c>
-      <c r="E50">
+      <c r="E95">
         <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!T6,NA())</f>
         <v/>
       </c>
-      <c r="F50">
+      <c r="F95">
         <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!I6,999)</f>
         <v/>
       </c>
-      <c r="G50">
+      <c r="G95">
         <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!X6,"")</f>
         <v/>
       </c>
-      <c r="H50">
+      <c r="H95">
         <f>IF(OR($B$4="Toutes",Data!AE6=$B$4),Data!Y6,0)</f>
         <v/>
       </c>
     </row>
-    <row r="51">
-      <c r="A51">
+    <row r="96">
+      <c r="A96">
         <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!A7,"")</f>
         <v/>
       </c>
-      <c r="B51">
+      <c r="B96">
         <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!D7,"")</f>
         <v/>
       </c>
-      <c r="C51">
+      <c r="C96">
         <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!H7,"")</f>
         <v/>
       </c>
-      <c r="D51">
+      <c r="D96">
         <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!Q7,"")</f>
         <v/>
       </c>
-      <c r="E51">
+      <c r="E96">
         <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!T7,NA())</f>
         <v/>
       </c>
-      <c r="F51">
+      <c r="F96">
         <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!I7,999)</f>
         <v/>
       </c>
-      <c r="G51">
+      <c r="G96">
         <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!X7,"")</f>
         <v/>
       </c>
-      <c r="H51">
+      <c r="H96">
         <f>IF(OR($B$4="Toutes",Data!AE7=$B$4),Data!Y7,0)</f>
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="A52">
+    <row r="97">
+      <c r="A97">
         <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!A8,"")</f>
         <v/>
       </c>
-      <c r="B52">
+      <c r="B97">
         <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!D8,"")</f>
         <v/>
       </c>
-      <c r="C52">
+      <c r="C97">
         <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!H8,"")</f>
         <v/>
       </c>
-      <c r="D52">
+      <c r="D97">
         <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!Q8,"")</f>
         <v/>
       </c>
-      <c r="E52">
+      <c r="E97">
         <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!T8,NA())</f>
         <v/>
       </c>
-      <c r="F52">
+      <c r="F97">
         <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!I8,999)</f>
         <v/>
       </c>
-      <c r="G52">
+      <c r="G97">
         <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!X8,"")</f>
         <v/>
       </c>
-      <c r="H52">
+      <c r="H97">
         <f>IF(OR($B$4="Toutes",Data!AE8=$B$4),Data!Y8,0)</f>
         <v/>
       </c>
     </row>
-    <row r="53">
-      <c r="A53">
+    <row r="98">
+      <c r="A98">
         <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!A9,"")</f>
         <v/>
       </c>
-      <c r="B53">
+      <c r="B98">
         <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!D9,"")</f>
         <v/>
       </c>
-      <c r="C53">
+      <c r="C98">
         <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!H9,"")</f>
         <v/>
       </c>
-      <c r="D53">
+      <c r="D98">
         <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!Q9,"")</f>
         <v/>
       </c>
-      <c r="E53">
+      <c r="E98">
         <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!T9,NA())</f>
         <v/>
       </c>
-      <c r="F53">
+      <c r="F98">
         <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!I9,999)</f>
         <v/>
       </c>
-      <c r="G53">
+      <c r="G98">
         <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!X9,"")</f>
         <v/>
       </c>
-      <c r="H53">
+      <c r="H98">
         <f>IF(OR($B$4="Toutes",Data!AE9=$B$4),Data!Y9,0)</f>
         <v/>
       </c>
     </row>
-    <row r="54">
-      <c r="A54">
+    <row r="99">
+      <c r="A99">
         <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!A10,"")</f>
         <v/>
       </c>
-      <c r="B54">
+      <c r="B99">
         <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!D10,"")</f>
         <v/>
       </c>
-      <c r="C54">
+      <c r="C99">
         <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!H10,"")</f>
         <v/>
       </c>
-      <c r="D54">
+      <c r="D99">
         <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!Q10,"")</f>
         <v/>
       </c>
-      <c r="E54">
+      <c r="E99">
         <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!T10,NA())</f>
         <v/>
       </c>
-      <c r="F54">
+      <c r="F99">
         <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!I10,999)</f>
         <v/>
       </c>
-      <c r="G54">
+      <c r="G99">
         <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!X10,"")</f>
         <v/>
       </c>
-      <c r="H54">
+      <c r="H99">
         <f>IF(OR($B$4="Toutes",Data!AE10=$B$4),Data!Y10,0)</f>
         <v/>
       </c>
     </row>
-    <row r="55">
-      <c r="A55">
+    <row r="100">
+      <c r="A100">
         <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!A11,"")</f>
         <v/>
       </c>
-      <c r="B55">
+      <c r="B100">
         <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!D11,"")</f>
         <v/>
       </c>
-      <c r="C55">
+      <c r="C100">
         <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!H11,"")</f>
         <v/>
       </c>
-      <c r="D55">
+      <c r="D100">
         <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!Q11,"")</f>
         <v/>
       </c>
-      <c r="E55">
+      <c r="E100">
         <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!T11,NA())</f>
         <v/>
       </c>
-      <c r="F55">
+      <c r="F100">
         <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!I11,999)</f>
         <v/>
       </c>
-      <c r="G55">
+      <c r="G100">
         <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!X11,"")</f>
         <v/>
       </c>
-      <c r="H55">
+      <c r="H100">
         <f>IF(OR($B$4="Toutes",Data!AE11=$B$4),Data!Y11,0)</f>
         <v/>
       </c>
     </row>
-    <row r="56">
-      <c r="A56">
+    <row r="101">
+      <c r="A101">
         <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!A12,"")</f>
         <v/>
       </c>
-      <c r="B56">
+      <c r="B101">
         <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!D12,"")</f>
         <v/>
       </c>
-      <c r="C56">
+      <c r="C101">
         <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!H12,"")</f>
         <v/>
       </c>
-      <c r="D56">
+      <c r="D101">
         <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!Q12,"")</f>
         <v/>
       </c>
-      <c r="E56">
+      <c r="E101">
         <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!T12,NA())</f>
         <v/>
       </c>
-      <c r="F56">
+      <c r="F101">
         <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!I12,999)</f>
         <v/>
       </c>
-      <c r="G56">
+      <c r="G101">
         <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!X12,"")</f>
         <v/>
       </c>
-      <c r="H56">
+      <c r="H101">
         <f>IF(OR($B$4="Toutes",Data!AE12=$B$4),Data!Y12,0)</f>
         <v/>
       </c>
     </row>
-    <row r="57">
-      <c r="A57">
+    <row r="102">
+      <c r="A102">
         <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!A13,"")</f>
         <v/>
       </c>
-      <c r="B57">
+      <c r="B102">
         <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!D13,"")</f>
         <v/>
       </c>
-      <c r="C57">
+      <c r="C102">
         <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!H13,"")</f>
         <v/>
       </c>
-      <c r="D57">
+      <c r="D102">
         <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!Q13,"")</f>
         <v/>
       </c>
-      <c r="E57">
+      <c r="E102">
         <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!T13,NA())</f>
         <v/>
       </c>
-      <c r="F57">
+      <c r="F102">
         <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!I13,999)</f>
         <v/>
       </c>
-      <c r="G57">
+      <c r="G102">
         <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!X13,"")</f>
         <v/>
       </c>
-      <c r="H57">
+      <c r="H102">
         <f>IF(OR($B$4="Toutes",Data!AE13=$B$4),Data!Y13,0)</f>
         <v/>
       </c>
     </row>
-    <row r="58">
-      <c r="A58">
+    <row r="103">
+      <c r="A103">
         <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!A14,"")</f>
         <v/>
       </c>
-      <c r="B58">
+      <c r="B103">
         <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!D14,"")</f>
         <v/>
       </c>
-      <c r="C58">
+      <c r="C103">
         <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!H14,"")</f>
         <v/>
       </c>
-      <c r="D58">
+      <c r="D103">
         <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!Q14,"")</f>
         <v/>
       </c>
-      <c r="E58">
+      <c r="E103">
         <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!T14,NA())</f>
         <v/>
       </c>
-      <c r="F58">
+      <c r="F103">
         <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!I14,999)</f>
         <v/>
       </c>
-      <c r="G58">
+      <c r="G103">
         <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!X14,"")</f>
         <v/>
       </c>
-      <c r="H58">
+      <c r="H103">
         <f>IF(OR($B$4="Toutes",Data!AE14=$B$4),Data!Y14,0)</f>
         <v/>
       </c>
     </row>
-    <row r="59">
-      <c r="A59">
+    <row r="104">
+      <c r="A104">
         <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!A15,"")</f>
         <v/>
       </c>
-      <c r="B59">
+      <c r="B104">
         <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!D15,"")</f>
         <v/>
       </c>
-      <c r="C59">
+      <c r="C104">
         <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!H15,"")</f>
         <v/>
       </c>
-      <c r="D59">
+      <c r="D104">
         <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!Q15,"")</f>
         <v/>
       </c>
-      <c r="E59">
+      <c r="E104">
         <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!T15,NA())</f>
         <v/>
       </c>
-      <c r="F59">
+      <c r="F104">
         <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!I15,999)</f>
         <v/>
       </c>
-      <c r="G59">
+      <c r="G104">
         <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!X15,"")</f>
         <v/>
       </c>
-      <c r="H59">
+      <c r="H104">
         <f>IF(OR($B$4="Toutes",Data!AE15=$B$4),Data!Y15,0)</f>
         <v/>
       </c>
     </row>
-    <row r="60">
-      <c r="A60">
+    <row r="105">
+      <c r="A105">
         <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!A16,"")</f>
         <v/>
       </c>
-      <c r="B60">
+      <c r="B105">
         <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!D16,"")</f>
         <v/>
       </c>
-      <c r="C60">
+      <c r="C105">
         <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!H16,"")</f>
         <v/>
       </c>
-      <c r="D60">
+      <c r="D105">
         <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!Q16,"")</f>
         <v/>
       </c>
-      <c r="E60">
+      <c r="E105">
         <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!T16,NA())</f>
         <v/>
       </c>
-      <c r="F60">
+      <c r="F105">
         <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!I16,999)</f>
         <v/>
       </c>
-      <c r="G60">
+      <c r="G105">
         <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!X16,"")</f>
         <v/>
       </c>
-      <c r="H60">
+      <c r="H105">
         <f>IF(OR($B$4="Toutes",Data!AE16=$B$4),Data!Y16,0)</f>
         <v/>
       </c>
     </row>
-    <row r="61">
-      <c r="A61">
+    <row r="106">
+      <c r="A106">
         <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!A17,"")</f>
         <v/>
       </c>
-      <c r="B61">
+      <c r="B106">
         <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!D17,"")</f>
         <v/>
       </c>
-      <c r="C61">
+      <c r="C106">
         <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!H17,"")</f>
         <v/>
       </c>
-      <c r="D61">
+      <c r="D106">
         <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!Q17,"")</f>
         <v/>
       </c>
-      <c r="E61">
+      <c r="E106">
         <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!T17,NA())</f>
         <v/>
       </c>
-      <c r="F61">
+      <c r="F106">
         <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!I17,999)</f>
         <v/>
       </c>
-      <c r="G61">
+      <c r="G106">
         <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!X17,"")</f>
         <v/>
       </c>
-      <c r="H61">
+      <c r="H106">
         <f>IF(OR($B$4="Toutes",Data!AE17=$B$4),Data!Y17,0)</f>
         <v/>
       </c>
     </row>
-    <row r="62">
-      <c r="A62">
+    <row r="107">
+      <c r="A107">
         <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!A18,"")</f>
         <v/>
       </c>
-      <c r="B62">
+      <c r="B107">
         <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!D18,"")</f>
         <v/>
       </c>
-      <c r="C62">
+      <c r="C107">
         <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!H18,"")</f>
         <v/>
       </c>
-      <c r="D62">
+      <c r="D107">
         <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!Q18,"")</f>
         <v/>
       </c>
-      <c r="E62">
+      <c r="E107">
         <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!T18,NA())</f>
         <v/>
       </c>
-      <c r="F62">
+      <c r="F107">
         <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!I18,999)</f>
         <v/>
       </c>
-      <c r="G62">
+      <c r="G107">
         <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!X18,"")</f>
         <v/>
       </c>
-      <c r="H62">
+      <c r="H107">
         <f>IF(OR($B$4="Toutes",Data!AE18=$B$4),Data!Y18,0)</f>
         <v/>
       </c>
     </row>
-    <row r="63">
-      <c r="A63">
+    <row r="108">
+      <c r="A108">
         <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!A19,"")</f>
         <v/>
       </c>
-      <c r="B63">
+      <c r="B108">
         <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!D19,"")</f>
         <v/>
       </c>
-      <c r="C63">
+      <c r="C108">
         <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!H19,"")</f>
         <v/>
       </c>
-      <c r="D63">
+      <c r="D108">
         <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!Q19,"")</f>
         <v/>
       </c>
-      <c r="E63">
+      <c r="E108">
         <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!T19,NA())</f>
         <v/>
       </c>
-      <c r="F63">
+      <c r="F108">
         <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!I19,999)</f>
         <v/>
       </c>
-      <c r="G63">
+      <c r="G108">
         <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!X19,"")</f>
         <v/>
       </c>
-      <c r="H63">
+      <c r="H108">
         <f>IF(OR($B$4="Toutes",Data!AE19=$B$4),Data!Y19,0)</f>
         <v/>
       </c>
@@ -4434,7 +4434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L43"/>
+  <dimension ref="A1:L103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4465,754 +4465,754 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>equipe</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B60" s="7" t="inlineStr">
         <is>
           <t>efficacite_offensive</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E60" s="7" t="inlineStr">
         <is>
           <t>equipe</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
+      <c r="F60" s="7" t="inlineStr">
         <is>
           <t>buts_encaisses</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t>Monaco</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B61" t="n">
         <v>1.1</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>PSG</t>
         </is>
       </c>
-      <c r="F6" t="n">
+      <c r="F61" t="n">
         <v>28</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="62">
+      <c r="A62" t="inlineStr">
         <is>
           <t>PSG</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B62" t="n">
         <v>1.08</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E62" t="inlineStr">
         <is>
           <t>Lille</t>
         </is>
       </c>
-      <c r="F7" t="n">
+      <c r="F62" t="n">
         <v>33</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="63">
+      <c r="A63" t="inlineStr">
         <is>
           <t>Marseille</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B63" t="n">
         <v>1.07</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>Nice</t>
         </is>
       </c>
-      <c r="F8" t="n">
+      <c r="F63" t="n">
         <v>34</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="64">
+      <c r="A64" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B64" t="n">
         <v>1.06</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>Marseille</t>
         </is>
       </c>
-      <c r="F9" t="n">
+      <c r="F64" t="n">
         <v>35</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="65">
+      <c r="A65" t="inlineStr">
         <is>
           <t>Lorient</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B65" t="n">
         <v>1.05</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E65" t="inlineStr">
         <is>
           <t>Lens</t>
         </is>
       </c>
-      <c r="F10" t="n">
+      <c r="F65" t="n">
         <v>38</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="66">
+      <c r="A66" t="inlineStr">
         <is>
           <t>Lille</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B66" t="n">
         <v>1.04</v>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>Monaco</t>
         </is>
       </c>
-      <c r="F11" t="n">
+      <c r="F66" t="n">
         <v>41</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="67">
+      <c r="A67" t="inlineStr">
         <is>
           <t>Rennes</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B67" t="n">
         <v>1.04</v>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="E67" t="inlineStr">
         <is>
           <t>Strasbourg</t>
         </is>
       </c>
-      <c r="F12" t="n">
+      <c r="F67" t="n">
         <v>42</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="68">
+      <c r="A68" t="inlineStr">
         <is>
           <t>Nice</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B68" t="n">
         <v>1.03</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E68" t="inlineStr">
         <is>
           <t>Brest</t>
         </is>
       </c>
-      <c r="F13" t="n">
+      <c r="F68" t="n">
         <v>43</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="69">
+      <c r="A69" t="inlineStr">
         <is>
           <t>Toulouse</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B69" t="n">
         <v>1.03</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E69" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="F14" t="n">
+      <c r="F69" t="n">
         <v>46</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
+    <row r="70">
+      <c r="A70" t="inlineStr">
         <is>
           <t>Brest</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B70" t="n">
         <v>1.03</v>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>Auxerre</t>
         </is>
       </c>
-      <c r="F15" t="n">
+      <c r="F70" t="n">
         <v>47</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="71">
+      <c r="A71" t="inlineStr">
         <is>
           <t>Auxerre</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B71" t="n">
         <v>1.01</v>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E71" t="inlineStr">
         <is>
           <t>Toulouse</t>
         </is>
       </c>
-      <c r="F16" t="n">
+      <c r="F71" t="n">
         <v>48</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="72">
+      <c r="A72" t="inlineStr">
         <is>
           <t>Strasbourg</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B72" t="n">
         <v>1</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E72" t="inlineStr">
         <is>
           <t>Angers</t>
         </is>
       </c>
-      <c r="F17" t="n">
+      <c r="F72" t="n">
         <v>49</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
+    <row r="73">
+      <c r="A73" t="inlineStr">
         <is>
           <t>Metz</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B73" t="n">
         <v>1</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="F18" t="n">
+      <c r="F73" t="n">
         <v>50</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="74">
+      <c r="A74" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B74" t="n">
         <v>0.99</v>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="E74" t="inlineStr">
         <is>
           <t>Rennes</t>
         </is>
       </c>
-      <c r="F19" t="n">
+      <c r="F74" t="n">
         <v>51</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
+    <row r="75">
+      <c r="A75" t="inlineStr">
         <is>
           <t>Lens</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B75" t="n">
         <v>0.98</v>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E75" t="inlineStr">
         <is>
           <t>Le Havre</t>
         </is>
       </c>
-      <c r="F20" t="n">
+      <c r="F75" t="n">
         <v>52</v>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
+    <row r="76">
+      <c r="A76" t="inlineStr">
         <is>
           <t>Angers</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B76" t="n">
         <v>0.98</v>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E76" t="inlineStr">
         <is>
           <t>Lorient</t>
         </is>
       </c>
-      <c r="F21" t="n">
+      <c r="F76" t="n">
         <v>57</v>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
+    <row r="77">
+      <c r="A77" t="inlineStr">
         <is>
           <t>Le Havre</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B77" t="n">
         <v>0.98</v>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>Metz</t>
         </is>
       </c>
-      <c r="F22" t="n">
+      <c r="F77" t="n">
         <v>60</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="78">
+      <c r="A78" t="inlineStr">
         <is>
           <t>Paris FC</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B78" t="n">
         <v>0.98</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E78" t="inlineStr">
         <is>
           <t>Paris FC</t>
         </is>
       </c>
-      <c r="F23" t="n">
+      <c r="F78" t="n">
         <v>63</v>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="7" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="7" t="inlineStr">
         <is>
           <t>equipe</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
+      <c r="B85" s="7" t="inlineStr">
         <is>
           <t>indice_discipline</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E85" s="7" t="inlineStr">
         <is>
           <t>equipe</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F85" s="7" t="inlineStr">
         <is>
           <t>points_domicile</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr">
+      <c r="G85" s="7" t="inlineStr">
         <is>
           <t>points_exterieur</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
+    <row r="86">
+      <c r="A86" t="inlineStr">
         <is>
           <t>Paris FC</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B86" t="n">
         <v>100</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>PSG</t>
         </is>
       </c>
-      <c r="F26" t="n">
+      <c r="F86" t="n">
         <v>43</v>
       </c>
-      <c r="G26" t="n">
+      <c r="G86" t="n">
         <v>39</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="87">
+      <c r="A87" t="inlineStr">
         <is>
           <t>Metz</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B87" t="n">
         <v>95</v>
       </c>
-      <c r="E27" t="inlineStr">
+      <c r="E87" t="inlineStr">
         <is>
           <t>Lille</t>
         </is>
       </c>
-      <c r="F27" t="n">
+      <c r="F87" t="n">
         <v>35</v>
       </c>
-      <c r="G27" t="n">
+      <c r="G87" t="n">
         <v>28</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="88">
+      <c r="A88" t="inlineStr">
         <is>
           <t>Lorient</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B88" t="n">
         <v>94</v>
       </c>
-      <c r="E28" t="inlineStr">
+      <c r="E88" t="inlineStr">
         <is>
           <t>Nice</t>
         </is>
       </c>
-      <c r="F28" t="n">
+      <c r="F88" t="n">
         <v>34</v>
       </c>
-      <c r="G28" t="n">
+      <c r="G88" t="n">
         <v>26</v>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="89">
+      <c r="A89" t="inlineStr">
         <is>
           <t>Le Havre</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="B89" t="n">
         <v>91</v>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E89" t="inlineStr">
         <is>
           <t>Marseille</t>
         </is>
       </c>
-      <c r="F29" t="n">
+      <c r="F89" t="n">
         <v>32</v>
       </c>
-      <c r="G29" t="n">
+      <c r="G89" t="n">
         <v>39</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="90">
+      <c r="A90" t="inlineStr">
         <is>
           <t>Auxerre</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B90" t="n">
         <v>85</v>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E90" t="inlineStr">
         <is>
           <t>Monaco</t>
         </is>
       </c>
-      <c r="F30" t="n">
+      <c r="F90" t="n">
         <v>31</v>
       </c>
-      <c r="G30" t="n">
+      <c r="G90" t="n">
         <v>37</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
+    <row r="91">
+      <c r="A91" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="B31" t="n">
+      <c r="B91" t="n">
         <v>85</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E91" t="inlineStr">
         <is>
           <t>Lens</t>
         </is>
       </c>
-      <c r="F31" t="n">
+      <c r="F91" t="n">
         <v>31</v>
       </c>
-      <c r="G31" t="n">
+      <c r="G91" t="n">
         <v>25</v>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
+    <row r="92">
+      <c r="A92" t="inlineStr">
         <is>
           <t>Angers</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B92" t="n">
         <v>84</v>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E92" t="inlineStr">
         <is>
           <t>Strasbourg</t>
         </is>
       </c>
-      <c r="F32" t="n">
+      <c r="F92" t="n">
         <v>30</v>
       </c>
-      <c r="G32" t="n">
+      <c r="G92" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="93">
+      <c r="A93" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B93" t="n">
         <v>82</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E93" t="inlineStr">
         <is>
           <t>Rennes</t>
         </is>
       </c>
-      <c r="F33" t="n">
+      <c r="F93" t="n">
         <v>28</v>
       </c>
-      <c r="G33" t="n">
+      <c r="G93" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
+    <row r="94">
+      <c r="A94" t="inlineStr">
         <is>
           <t>Rennes</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B94" t="n">
         <v>80</v>
       </c>
-      <c r="E34" t="inlineStr">
+      <c r="E94" t="inlineStr">
         <is>
           <t>Lyon</t>
         </is>
       </c>
-      <c r="F34" t="n">
+      <c r="F94" t="n">
         <v>26</v>
       </c>
-      <c r="G34" t="n">
+      <c r="G94" t="n">
         <v>32</v>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="95">
+      <c r="A95" t="inlineStr">
         <is>
           <t>Strasbourg</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B95" t="n">
         <v>78</v>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E95" t="inlineStr">
         <is>
           <t>Toulouse</t>
         </is>
       </c>
-      <c r="F35" t="n">
+      <c r="F95" t="n">
         <v>26</v>
       </c>
-      <c r="G35" t="n">
+      <c r="G95" t="n">
         <v>21</v>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
+    <row r="96">
+      <c r="A96" t="inlineStr">
         <is>
           <t>Lens</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B96" t="n">
         <v>77</v>
       </c>
-      <c r="E36" t="inlineStr">
+      <c r="E96" t="inlineStr">
         <is>
           <t>Auxerre</t>
         </is>
       </c>
-      <c r="F36" t="n">
+      <c r="F96" t="n">
         <v>25</v>
       </c>
-      <c r="G36" t="n">
+      <c r="G96" t="n">
         <v>20</v>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="97">
+      <c r="A97" t="inlineStr">
         <is>
           <t>Marseille</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B97" t="n">
         <v>73</v>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E97" t="inlineStr">
         <is>
           <t>Brest</t>
         </is>
       </c>
-      <c r="F37" t="n">
+      <c r="F97" t="n">
         <v>22</v>
       </c>
-      <c r="G37" t="n">
+      <c r="G97" t="n">
         <v>29</v>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
+    <row r="98">
+      <c r="A98" t="inlineStr">
         <is>
           <t>Toulouse</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B98" t="n">
         <v>73</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E98" t="inlineStr">
         <is>
           <t>Angers</t>
         </is>
       </c>
-      <c r="F38" t="n">
+      <c r="F98" t="n">
         <v>22</v>
       </c>
-      <c r="G38" t="n">
+      <c r="G98" t="n">
         <v>18</v>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
+    <row r="99">
+      <c r="A99" t="inlineStr">
         <is>
           <t>Nice</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B99" t="n">
         <v>72</v>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E99" t="inlineStr">
         <is>
           <t>Le Havre</t>
         </is>
       </c>
-      <c r="F39" t="n">
+      <c r="F99" t="n">
         <v>21</v>
       </c>
-      <c r="G39" t="n">
+      <c r="G99" t="n">
         <v>17</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
+    <row r="100">
+      <c r="A100" t="inlineStr">
         <is>
           <t>Brest</t>
         </is>
       </c>
-      <c r="B40" t="n">
+      <c r="B100" t="n">
         <v>71</v>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E100" t="inlineStr">
         <is>
           <t>Lorient</t>
         </is>
       </c>
-      <c r="F40" t="n">
+      <c r="F100" t="n">
         <v>20</v>
       </c>
-      <c r="G40" t="n">
+      <c r="G100" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="101">
+      <c r="A101" t="inlineStr">
         <is>
           <t>Monaco</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="B101" t="n">
         <v>67</v>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E101" t="inlineStr">
         <is>
           <t>Nantes</t>
         </is>
       </c>
-      <c r="F41" t="n">
+      <c r="F101" t="n">
         <v>18</v>
       </c>
-      <c r="G41" t="n">
+      <c r="G101" t="n">
         <v>24</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
+    <row r="102">
+      <c r="A102" t="inlineStr">
         <is>
           <t>PSG</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B102" t="n">
         <v>64</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E102" t="inlineStr">
         <is>
           <t>Metz</t>
         </is>
       </c>
-      <c r="F42" t="n">
+      <c r="F102" t="n">
         <v>18</v>
       </c>
-      <c r="G42" t="n">
+      <c r="G102" t="n">
         <v>13</v>
       </c>
     </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
+    <row r="103">
+      <c r="A103" t="inlineStr">
         <is>
           <t>Lille</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B103" t="n">
         <v>60</v>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E103" t="inlineStr">
         <is>
           <t>Paris FC</t>
         </is>
       </c>
-      <c r="F43" t="n">
+      <c r="F103" t="n">
         <v>16</v>
       </c>
-      <c r="G43" t="n">
+      <c r="G103" t="n">
         <v>12</v>
       </c>
     </row>

</xml_diff>